<commit_message>
adding data + gov
</commit_message>
<xml_diff>
--- a/data/input/department_tracking.xlsx
+++ b/data/input/department_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ADriscoll/Documents/GitHub/implied_data/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4824C945-A7AE-724A-B5EB-8079EF6B6537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C7D9B6-286F-6048-80C0-BCD00DE9DBA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="27180" windowHeight="17060" xr2:uid="{484B642E-F565-954E-B324-BC6070DF60AE}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17060" xr2:uid="{484B642E-F565-954E-B324-BC6070DF60AE}"/>
   </bookViews>
   <sheets>
     <sheet name="letters" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="250">
   <si>
     <t>type</t>
   </si>
@@ -342,9 +342,6 @@
     <t xml:space="preserve">Center for Innovation through Data Intelligence </t>
   </si>
   <si>
-    <t xml:space="preserve">City Commission on Human Rights </t>
-  </si>
-  <si>
     <t xml:space="preserve">Civic Engagement Commission </t>
   </si>
   <si>
@@ -708,9 +705,6 @@
     <t>MOPD</t>
   </si>
   <si>
-    <t>Office of Talent and Workforce Development</t>
-  </si>
-  <si>
     <t>NYC Talent</t>
   </si>
   <si>
@@ -741,9 +735,6 @@
     <t>Erik</t>
   </si>
   <si>
-    <t>include 2</t>
-  </si>
-  <si>
     <t>Brook</t>
   </si>
   <si>
@@ -757,13 +748,55 @@
   </si>
   <si>
     <t>DSS (HRA + DHS)</t>
+  </si>
+  <si>
+    <t>Ending Gender Based Violence</t>
+  </si>
+  <si>
+    <t>combine</t>
+  </si>
+  <si>
+    <t>charter</t>
+  </si>
+  <si>
+    <t>adcode</t>
+  </si>
+  <si>
+    <t>rules</t>
+  </si>
+  <si>
+    <t>People with Disabilities</t>
+  </si>
+  <si>
+    <t>Community Mental Health</t>
+  </si>
+  <si>
+    <t>Criminal Justice</t>
+  </si>
+  <si>
+    <t>Economic Development Cooperation</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office of </t>
+  </si>
+  <si>
+    <t>Talent and Workforce Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Human Rights </t>
+  </si>
+  <si>
+    <t>City Commission on</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -782,6 +815,13 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -805,16 +845,57 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1155,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03E8848C-B962-5745-8655-3C2761762076}">
-  <dimension ref="A1:K54"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
@@ -1163,20 +1244,21 @@
     <col min="3" max="3" width="14.5" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" customWidth="1"/>
+    <col min="8" max="11" width="8.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>86</v>
+        <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>88</v>
@@ -1188,27 +1270,33 @@
         <v>2</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>3</v>
+        <v>239</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>160</v>
+        <v>240</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C2" t="s">
+        <v>209</v>
       </c>
       <c r="D2">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -1217,520 +1305,496 @@
         <v>80</v>
       </c>
       <c r="G2">
-        <v>0.33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>206</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
+        <v>172</v>
       </c>
       <c r="D3">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E3">
         <v>1</v>
       </c>
       <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B4" t="s">
+        <v>224</v>
+      </c>
+      <c r="C4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D4">
+        <v>9</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
         <v>80</v>
       </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" t="s">
-        <v>110</v>
-      </c>
-      <c r="C4" t="s">
-        <v>166</v>
-      </c>
-      <c r="D4">
-        <v>10</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
-        <v>82</v>
-      </c>
       <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4" s="3">
-        <v>46156</v>
-      </c>
-      <c r="I4" t="s">
-        <v>234</v>
-      </c>
-      <c r="J4" t="s">
-        <v>235</v>
-      </c>
-      <c r="K4" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5">
+        <v>5</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>82</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6">
+        <v>5</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+      <c r="F6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>236</v>
+      </c>
+      <c r="B8" t="s">
+        <v>114</v>
+      </c>
+      <c r="C8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>80</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B9" t="s">
+        <v>109</v>
+      </c>
+      <c r="C9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
+        <v>82</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" t="s">
+        <v>215</v>
+      </c>
+      <c r="D10">
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>80</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>244</v>
+      </c>
+      <c r="B11" t="s">
+        <v>245</v>
+      </c>
+      <c r="C11" t="s">
+        <v>217</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>247</v>
+      </c>
+      <c r="B12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C12" t="s">
+        <v>221</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12" t="s">
+        <v>81</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" t="s">
         <v>112</v>
       </c>
-      <c r="C5" t="s">
-        <v>153</v>
-      </c>
-      <c r="D5">
-        <v>10</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-      <c r="I5" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" t="s">
-        <v>238</v>
-      </c>
-      <c r="D6">
-        <v>10</v>
-      </c>
-      <c r="E6">
-        <v>1</v>
-      </c>
-      <c r="F6" t="s">
-        <v>82</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-      <c r="H6" s="3">
-        <v>46156</v>
-      </c>
-      <c r="I6" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C7" t="s">
-        <v>210</v>
-      </c>
-      <c r="D7">
-        <v>10</v>
-      </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
+      <c r="C13" t="s">
+        <v>193</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B14" t="s">
+        <v>114</v>
+      </c>
+      <c r="C14" t="s">
+        <v>219</v>
+      </c>
+      <c r="D14">
+        <v>3</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C8" t="s">
-        <v>165</v>
-      </c>
-      <c r="D8">
-        <v>9</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>82</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" t="s">
-        <v>130</v>
-      </c>
-      <c r="D9">
-        <v>9</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
-        <v>82</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>67</v>
-      </c>
-      <c r="B10" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" t="s">
-        <v>173</v>
-      </c>
-      <c r="D10">
-        <v>9</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>82</v>
-      </c>
-      <c r="G10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B11" t="s">
-        <v>111</v>
-      </c>
-      <c r="C11" t="s">
-        <v>176</v>
-      </c>
-      <c r="D11">
-        <v>9</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11" t="s">
-        <v>82</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>227</v>
-      </c>
-      <c r="B12" t="s">
-        <v>226</v>
-      </c>
-      <c r="C12" t="s">
-        <v>225</v>
-      </c>
-      <c r="D12">
-        <v>9</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="G12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B13" t="s">
-        <v>111</v>
-      </c>
-      <c r="C13" t="s">
-        <v>183</v>
-      </c>
-      <c r="D13">
-        <v>8</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
-        <v>82</v>
-      </c>
-      <c r="G13">
-        <v>0</v>
-      </c>
-      <c r="I13" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" t="s">
-        <v>182</v>
-      </c>
-      <c r="D14">
-        <v>8</v>
-      </c>
-      <c r="E14">
-        <v>1</v>
-      </c>
-      <c r="F14" t="s">
-        <v>82</v>
-      </c>
       <c r="G14">
         <v>0</v>
       </c>
-      <c r="I14" t="s">
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>242</v>
+      </c>
+      <c r="B15" t="s">
+        <v>114</v>
+      </c>
+      <c r="C15" t="s">
+        <v>222</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15" t="s">
+        <v>81</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>248</v>
+      </c>
+      <c r="B16" t="s">
+        <v>249</v>
+      </c>
+      <c r="C16" t="s">
+        <v>139</v>
+      </c>
+      <c r="D16">
+        <v>2</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16">
+        <v>0</v>
+      </c>
+      <c r="L16" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" t="s">
-        <v>110</v>
-      </c>
-      <c r="C15" t="s">
-        <v>168</v>
-      </c>
-      <c r="D15">
-        <v>8</v>
-      </c>
-      <c r="E15">
-        <v>1</v>
-      </c>
-      <c r="F15" t="s">
-        <v>82</v>
-      </c>
-      <c r="G15">
-        <v>0</v>
-      </c>
-      <c r="I15" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" t="s">
-        <v>110</v>
-      </c>
-      <c r="C16" t="s">
-        <v>151</v>
-      </c>
-      <c r="D16">
-        <v>7</v>
-      </c>
-      <c r="E16">
-        <v>1</v>
-      </c>
-      <c r="F16" t="s">
-        <v>82</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-      <c r="I16" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
         <v>114</v>
       </c>
       <c r="C17" t="s">
+        <v>202</v>
+      </c>
+      <c r="D17">
+        <v>2</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>241</v>
+      </c>
+      <c r="B18" t="s">
+        <v>114</v>
+      </c>
+      <c r="C18" t="s">
+        <v>220</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="D17">
+      <c r="D19">
+        <v>99</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="D20">
+        <v>99</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" t="s">
+        <v>158</v>
+      </c>
+      <c r="D21">
         <v>7</v>
       </c>
-      <c r="E17">
-        <v>1</v>
-      </c>
-      <c r="F17" t="s">
-        <v>82</v>
-      </c>
-      <c r="G17">
+      <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s">
+        <v>82</v>
+      </c>
+      <c r="G21">
         <v>0.66</v>
       </c>
-      <c r="I17" t="s">
-        <v>236</v>
-      </c>
-      <c r="J17" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+      <c r="L21" t="s">
+        <v>233</v>
+      </c>
+      <c r="M21" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>11</v>
       </c>
-      <c r="B18" t="s">
-        <v>110</v>
-      </c>
-      <c r="C18" t="s">
-        <v>155</v>
-      </c>
-      <c r="D18">
+      <c r="B22" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" t="s">
+        <v>154</v>
+      </c>
+      <c r="D22">
         <v>7</v>
       </c>
-      <c r="E18">
-        <v>1</v>
-      </c>
-      <c r="F18" t="s">
-        <v>82</v>
-      </c>
-      <c r="G18">
+      <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22">
         <v>0.66</v>
       </c>
-      <c r="I18" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" t="s">
-        <v>110</v>
-      </c>
-      <c r="C19" t="s">
-        <v>164</v>
-      </c>
-      <c r="D19">
-        <v>7</v>
-      </c>
-      <c r="E19">
-        <v>1</v>
-      </c>
-      <c r="F19" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+      <c r="L22" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="s">
-        <v>110</v>
-      </c>
-      <c r="C20" t="s">
-        <v>157</v>
-      </c>
-      <c r="D20">
+      <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
+        <v>156</v>
+      </c>
+      <c r="D23">
         <v>6</v>
-      </c>
-      <c r="E20">
-        <v>1</v>
-      </c>
-      <c r="F20" t="s">
-        <v>82</v>
-      </c>
-      <c r="G20">
-        <v>0.66</v>
-      </c>
-      <c r="I20" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>62</v>
-      </c>
-      <c r="B21" t="s">
-        <v>110</v>
-      </c>
-      <c r="C21" t="s">
-        <v>154</v>
-      </c>
-      <c r="D21">
-        <v>6</v>
-      </c>
-      <c r="E21">
-        <v>1</v>
-      </c>
-      <c r="F21" t="s">
-        <v>82</v>
-      </c>
-      <c r="G21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22" t="s">
-        <v>111</v>
-      </c>
-      <c r="C22" t="s">
-        <v>152</v>
-      </c>
-      <c r="D22">
-        <v>6</v>
-      </c>
-      <c r="E22">
-        <v>1</v>
-      </c>
-      <c r="F22" t="s">
-        <v>82</v>
-      </c>
-      <c r="G22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>76</v>
-      </c>
-      <c r="B23" t="s">
-        <v>113</v>
-      </c>
-      <c r="C23" t="s">
-        <v>158</v>
-      </c>
-      <c r="D23">
-        <v>5</v>
       </c>
       <c r="E23">
         <v>1</v>
@@ -1741,19 +1805,19 @@
       <c r="G23">
         <v>0.66</v>
       </c>
-      <c r="I23" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="L23" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C24" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D24">
         <v>5</v>
@@ -1765,21 +1829,24 @@
         <v>82</v>
       </c>
       <c r="G24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+        <v>0.66</v>
+      </c>
+      <c r="L24" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C25" t="s">
-        <v>178</v>
+        <v>155</v>
       </c>
       <c r="D25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E25">
         <v>1</v>
@@ -1788,21 +1855,21 @@
         <v>82</v>
       </c>
       <c r="G25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="B26" t="s">
         <v>109</v>
       </c>
       <c r="C26" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="D26">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E26">
         <v>1</v>
@@ -1813,36 +1880,67 @@
       <c r="G26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H26" s="3">
+        <v>46156</v>
+      </c>
+      <c r="I26" s="3">
+        <v>46156</v>
+      </c>
+      <c r="J26" s="3">
+        <v>46156</v>
+      </c>
+      <c r="K26" s="3">
+        <v>46156</v>
+      </c>
+      <c r="L26" t="s">
+        <v>231</v>
+      </c>
+      <c r="M26" t="s">
+        <v>232</v>
+      </c>
+      <c r="N26" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>29</v>
+        <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="C27" t="s">
-        <v>188</v>
+        <v>235</v>
       </c>
       <c r="D27">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E27">
         <v>1</v>
       </c>
       <c r="F27" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="G27">
-        <v>0</v>
-      </c>
-      <c r="I27" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" t="s">
+        <v>109</v>
+      </c>
       <c r="C28" t="s">
-        <v>219</v>
+        <v>174</v>
       </c>
       <c r="D28">
         <v>4</v>
@@ -1850,25 +1948,37 @@
       <c r="E28">
         <v>1</v>
       </c>
+      <c r="F28" t="s">
+        <v>82</v>
+      </c>
       <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="I28" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H28" s="3">
+        <v>46161</v>
+      </c>
+      <c r="I28" s="3">
+        <v>46161</v>
+      </c>
+      <c r="J28" s="3">
+        <v>46161</v>
+      </c>
+      <c r="K28" s="3">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C29" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D29">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E29">
         <v>1</v>
@@ -1877,21 +1987,27 @@
         <v>82</v>
       </c>
       <c r="G29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H29" s="3">
+        <v>46161</v>
+      </c>
+      <c r="I29" s="3">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>89</v>
       </c>
       <c r="B30" t="s">
-        <v>110</v>
+        <v>245</v>
       </c>
       <c r="C30" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="D30">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E30">
         <v>1</v>
@@ -1902,19 +2018,25 @@
       <c r="G30">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H30" s="3">
+        <v>46161</v>
+      </c>
+      <c r="I30" s="3">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B31" t="s">
         <v>110</v>
       </c>
       <c r="C31" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E31">
         <v>1</v>
@@ -1923,44 +2045,59 @@
         <v>82</v>
       </c>
       <c r="G31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H31" s="3">
+        <v>46161</v>
+      </c>
+      <c r="I31" s="3">
+        <v>46161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="B32" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C32" t="s">
-        <v>216</v>
+        <v>182</v>
       </c>
       <c r="D32">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E32">
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H32" s="3">
+        <v>46161</v>
+      </c>
+      <c r="I32" s="3">
+        <v>46161</v>
+      </c>
+      <c r="L32" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>71</v>
+        <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C33" t="s">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="D33">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -1969,12 +2106,24 @@
         <v>82</v>
       </c>
       <c r="G33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H33" s="3">
+        <v>46162</v>
+      </c>
+      <c r="I33" s="3">
+        <v>46162</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>21</v>
+      </c>
+      <c r="B34" t="s">
+        <v>109</v>
+      </c>
       <c r="C34" t="s">
-        <v>218</v>
+        <v>161</v>
       </c>
       <c r="D34">
         <v>4</v>
@@ -1982,171 +2131,257 @@
       <c r="E34">
         <v>1</v>
       </c>
+      <c r="F34" t="s">
+        <v>82</v>
+      </c>
       <c r="G34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+        <v>1</v>
+      </c>
+      <c r="H34" s="3">
+        <v>46163</v>
+      </c>
+      <c r="I34" s="3">
+        <v>46163</v>
+      </c>
+      <c r="J34" s="3">
+        <v>46163</v>
+      </c>
+      <c r="K34" s="3">
+        <v>46163</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>222</v>
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>111</v>
       </c>
       <c r="C35" t="s">
-        <v>223</v>
+        <v>152</v>
       </c>
       <c r="D35">
+        <v>10</v>
+      </c>
+      <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35" t="s">
+        <v>82</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35" s="3">
+        <v>46163</v>
+      </c>
+      <c r="I35" s="3">
+        <v>46163</v>
+      </c>
+      <c r="L35" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" t="s">
+        <v>119</v>
+      </c>
+      <c r="C36" t="s">
+        <v>181</v>
+      </c>
+      <c r="D36">
+        <v>8</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36" t="s">
+        <v>82</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="L36" t="s">
+        <v>227</v>
+      </c>
+      <c r="M36" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37" t="s">
+        <v>109</v>
+      </c>
+      <c r="C37" t="s">
+        <v>167</v>
+      </c>
+      <c r="D37">
+        <v>8</v>
+      </c>
+      <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37" t="s">
+        <v>82</v>
+      </c>
+      <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="L37" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s">
+        <v>109</v>
+      </c>
+      <c r="C38" t="s">
+        <v>150</v>
+      </c>
+      <c r="D38">
+        <v>7</v>
+      </c>
+      <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38" t="s">
+        <v>82</v>
+      </c>
+      <c r="G38">
+        <v>1</v>
+      </c>
+      <c r="L38" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" t="s">
+        <v>109</v>
+      </c>
+      <c r="C39" t="s">
+        <v>153</v>
+      </c>
+      <c r="D39">
+        <v>6</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" t="s">
+        <v>82</v>
+      </c>
+      <c r="G39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" t="s">
+        <v>110</v>
+      </c>
+      <c r="C40" t="s">
+        <v>151</v>
+      </c>
+      <c r="D40">
+        <v>6</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40" t="s">
+        <v>82</v>
+      </c>
+      <c r="G40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>10</v>
+      </c>
+      <c r="B41" t="s">
+        <v>108</v>
+      </c>
+      <c r="C41" t="s">
+        <v>148</v>
+      </c>
+      <c r="D41">
+        <v>5</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" t="s">
+        <v>82</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>27</v>
+      </c>
+      <c r="B42" t="s">
+        <v>109</v>
+      </c>
+      <c r="C42" t="s">
+        <v>149</v>
+      </c>
+      <c r="D42">
         <v>4</v>
       </c>
-      <c r="E35">
-        <v>1</v>
-      </c>
-      <c r="G35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" t="s">
-        <v>110</v>
-      </c>
-      <c r="C36" t="s">
-        <v>156</v>
-      </c>
-      <c r="D36">
-        <v>3</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" t="s">
-        <v>82</v>
-      </c>
-      <c r="G36">
-        <v>0.66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A37" t="s">
-        <v>56</v>
-      </c>
-      <c r="B37" t="s">
-        <v>113</v>
-      </c>
-      <c r="C37" t="s">
-        <v>194</v>
-      </c>
-      <c r="D37">
-        <v>3</v>
-      </c>
-      <c r="E37">
-        <v>1</v>
-      </c>
-      <c r="F37" t="s">
-        <v>81</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C38" t="s">
-        <v>220</v>
-      </c>
-      <c r="D38">
-        <v>3</v>
-      </c>
-      <c r="E38">
-        <v>1</v>
-      </c>
-      <c r="G38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C39" t="s">
-        <v>224</v>
-      </c>
-      <c r="D39">
-        <v>3</v>
-      </c>
-      <c r="E39">
-        <v>1</v>
-      </c>
-      <c r="G39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>100</v>
-      </c>
-      <c r="C40" t="s">
-        <v>140</v>
-      </c>
-      <c r="D40">
-        <v>2</v>
-      </c>
-      <c r="E40">
-        <v>1</v>
-      </c>
-      <c r="F40" t="s">
-        <v>84</v>
-      </c>
-      <c r="G40">
-        <v>0</v>
-      </c>
-      <c r="I40" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A41" t="s">
-        <v>23</v>
-      </c>
-      <c r="B41" t="s">
-        <v>115</v>
-      </c>
-      <c r="C41" t="s">
-        <v>203</v>
-      </c>
-      <c r="D41">
-        <v>2</v>
-      </c>
-      <c r="E41">
-        <v>1</v>
-      </c>
-      <c r="F41" t="s">
-        <v>80</v>
-      </c>
-      <c r="G41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="C42" t="s">
-        <v>221</v>
-      </c>
-      <c r="D42">
-        <v>2</v>
-      </c>
       <c r="E42">
         <v>1</v>
       </c>
+      <c r="F42" t="s">
+        <v>82</v>
+      </c>
       <c r="G42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="6:6" x14ac:dyDescent="0.2">
-      <c r="F54" s="2"/>
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K55">
-    <sortCondition descending="1" ref="D1:D55"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N42">
+    <sortCondition ref="G1:G42"/>
   </sortState>
-  <conditionalFormatting sqref="H1:H1048576">
+  <conditionalFormatting sqref="K1 K3:K33 H26:J28 K35:K1048576">
+    <cfRule type="containsBlanks" dxfId="4" priority="7">
+      <formula>LEN(TRIM(H1))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:K2 H3:J25 J29:J32 H33:J42">
+    <cfRule type="containsBlanks" dxfId="3" priority="4">
+      <formula>LEN(TRIM(H2))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H29:H32">
+    <cfRule type="containsBlanks" dxfId="2" priority="3">
+      <formula>LEN(TRIM(H29))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I29:I32">
+    <cfRule type="containsBlanks" dxfId="1" priority="2">
+      <formula>LEN(TRIM(I29))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K34">
     <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(H1))=0</formula>
+      <formula>LEN(TRIM(K34))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2184,7 +2419,7 @@
         <v>86</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>88</v>
@@ -2204,10 +2439,10 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E3" t="s">
         <v>81</v>
@@ -2218,7 +2453,7 @@
         <v>98</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E4" t="s">
         <v>84</v>
@@ -2229,10 +2464,10 @@
         <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C5" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E5" t="s">
         <v>85</v>
@@ -2243,10 +2478,10 @@
         <v>66</v>
       </c>
       <c r="B6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E6" t="s">
         <v>82</v>
@@ -2260,10 +2495,10 @@
         <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E7" t="s">
         <v>84</v>
@@ -2271,10 +2506,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E8" t="s">
         <v>85</v>
@@ -2282,10 +2517,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E9" t="s">
         <v>84</v>
@@ -2296,10 +2531,10 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E10" t="s">
         <v>80</v>
@@ -2310,7 +2545,7 @@
         <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E11" t="s">
         <v>83</v>
@@ -2324,10 +2559,10 @@
         <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C12" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E12" t="s">
         <v>84</v>
@@ -2338,7 +2573,7 @@
         <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E13" t="s">
         <v>84</v>
@@ -2346,10 +2581,10 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C14" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>85</v>
@@ -2360,10 +2595,10 @@
         <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C15" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="E15" t="s">
         <v>84</v>
@@ -2371,10 +2606,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E16" t="s">
         <v>84</v>
@@ -2385,7 +2620,7 @@
         <v>93</v>
       </c>
       <c r="C17" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E17" t="s">
         <v>82</v>
@@ -2399,10 +2634,10 @@
         <v>48</v>
       </c>
       <c r="B18" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E18" t="s">
         <v>82</v>
@@ -2416,10 +2651,10 @@
         <v>55</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E19" t="s">
         <v>82</v>
@@ -2433,10 +2668,10 @@
         <v>69</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E20" t="s">
         <v>82</v>
@@ -2447,10 +2682,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E21" t="s">
         <v>84</v>
@@ -2461,7 +2696,7 @@
         <v>95</v>
       </c>
       <c r="C22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E22" t="s">
         <v>82</v>
@@ -2475,10 +2710,10 @@
         <v>46</v>
       </c>
       <c r="B23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C23" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E23" t="s">
         <v>82</v>
@@ -2492,7 +2727,7 @@
         <v>94</v>
       </c>
       <c r="C24" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E24" t="s">
         <v>82</v>
@@ -2506,10 +2741,10 @@
         <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C25" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E25" t="s">
         <v>80</v>
@@ -2520,7 +2755,7 @@
         <v>90</v>
       </c>
       <c r="C26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E26" t="s">
         <v>82</v>
@@ -2534,7 +2769,7 @@
         <v>92</v>
       </c>
       <c r="C27" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E27" t="s">
         <v>83</v>
@@ -2548,10 +2783,10 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C28" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E28" t="s">
         <v>80</v>
@@ -2562,10 +2797,10 @@
         <v>38</v>
       </c>
       <c r="B29" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="E29" t="s">
         <v>80</v>
@@ -2576,10 +2811,10 @@
         <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C30" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="E30" t="s">
         <v>80</v>
@@ -2590,10 +2825,10 @@
         <v>40</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="E31" t="s">
         <v>80</v>
@@ -2604,10 +2839,10 @@
         <v>44</v>
       </c>
       <c r="B32" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C32" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E32" t="s">
         <v>80</v>
@@ -2618,10 +2853,10 @@
         <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E33" t="s">
         <v>81</v>
@@ -2632,10 +2867,10 @@
         <v>59</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C34" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="E34" t="s">
         <v>80</v>
@@ -2646,10 +2881,10 @@
         <v>61</v>
       </c>
       <c r="B35" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C35" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E35" t="s">
         <v>80</v>
@@ -2660,10 +2895,10 @@
         <v>60</v>
       </c>
       <c r="B36" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C36" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E36" t="s">
         <v>80</v>
@@ -2674,7 +2909,7 @@
         <v>96</v>
       </c>
       <c r="C37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E37" t="s">
         <v>82</v>
@@ -2688,10 +2923,10 @@
         <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C38" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="E38" t="s">
         <v>80</v>
@@ -2702,10 +2937,10 @@
         <v>19</v>
       </c>
       <c r="B39" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
@@ -2713,10 +2948,10 @@
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C40" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="E40" t="s">
         <v>82</v>
@@ -2730,10 +2965,10 @@
         <v>49</v>
       </c>
       <c r="B41" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C41" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E41" t="s">
         <v>82</v>
@@ -2747,10 +2982,10 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C42" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E42" t="s">
         <v>81</v>
@@ -2761,10 +2996,10 @@
         <v>66</v>
       </c>
       <c r="B43" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C43" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E43" t="s">
         <v>82</v>
@@ -2778,10 +3013,10 @@
         <v>8</v>
       </c>
       <c r="B44" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C44" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E44" t="s">
         <v>81</v>
@@ -2792,10 +3027,10 @@
         <v>9</v>
       </c>
       <c r="B45" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C45" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E45" t="s">
         <v>83</v>
@@ -2809,10 +3044,10 @@
         <v>13</v>
       </c>
       <c r="B46" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C46" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E46" t="s">
         <v>80</v>
@@ -2823,10 +3058,10 @@
         <v>12</v>
       </c>
       <c r="B47" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C47" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E47" t="s">
         <v>81</v>
@@ -2837,10 +3072,10 @@
         <v>31</v>
       </c>
       <c r="B48" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C48" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="E48" t="s">
         <v>81</v>
@@ -2851,10 +3086,10 @@
         <v>42</v>
       </c>
       <c r="B49" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C49" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E49" t="s">
         <v>80</v>
@@ -2865,10 +3100,10 @@
         <v>53</v>
       </c>
       <c r="B50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C50" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E50" t="s">
         <v>81</v>
@@ -2879,10 +3114,10 @@
         <v>63</v>
       </c>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="E51" t="s">
         <v>81</v>
@@ -2890,10 +3125,10 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C52" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E52" t="s">
         <v>84</v>
@@ -2901,10 +3136,10 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C53" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E53" t="s">
         <v>85</v>
@@ -2915,10 +3150,10 @@
         <v>66</v>
       </c>
       <c r="B54" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C54" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="E54" t="s">
         <v>82</v>
@@ -2929,10 +3164,10 @@
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C55" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E55" t="s">
         <v>85</v>
@@ -2943,10 +3178,10 @@
         <v>74</v>
       </c>
       <c r="B56" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C56" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E56" t="s">
         <v>82</v>

</xml_diff>